<commit_message>
S42: Add Job ID column to upload template
Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/data/slotops_upload_template.xlsx
+++ b/data/slotops_upload_template.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -515,17 +515,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Client Name</t>
+          <t>Job ID</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>REQUIRED</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Your client or company name (e.g., Taskify, QuikHire)</t>
+          <t>Unique job identifier (e.g., JOB-001, LinkedIn Job ID). Auto-generated if blank.</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Job Title</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -559,31 +559,31 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Full country name or 2-letter code (US, GB, IN, DE, etc.)</t>
+          <t>The job title exactly as it appears on LinkedIn</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>REQUIRED</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>City name (e.g., New York, London, Mumbai)</t>
+          <t>Full country name or 2-letter code (US, GB, IN, DE, etc.)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>State/Region</t>
+          <t>City</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -593,14 +593,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>State code (NY, TX, CA) or region</t>
+          <t>City name (e.g., New York, London, Mumbai)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Job Function</t>
+          <t>State/Region</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -610,14 +610,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Engineering, Healthcare, Sales, Marketing, etc.</t>
+          <t>State code (NY, TX, CA) or region</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Job Function</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -627,14 +627,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Technology, Healthcare, Retail, Financial Services, etc.</t>
+          <t>Engineering, Healthcare, Sales, Marketing, etc.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Workplace Type</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -644,14 +644,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Remote, Hybrid, or On-site (default: Remote)</t>
+          <t>Technology, Healthcare, Retail, Financial Services, etc.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Application Method</t>
+          <t>Workplace Type</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -661,14 +661,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Easy Apply or ATS (default: ATS). Easy Apply gets 2.3x more applies!</t>
+          <t>Remote, Hybrid, or On-site (default: Remote)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Job URL</t>
+          <t>Application Method</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -678,14 +678,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Link to the job posting</t>
+          <t>Easy Apply or ATS (default: ATS). Easy Apply gets 2.3x more applies!</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Reference Number</t>
+          <t>Job URL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -695,14 +695,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Your internal reference/tracking number</t>
+          <t>Link to the job posting</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Reference Number</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -712,27 +712,45 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>High, Medium, or Low (default: Medium)</t>
+          <t>Your internal reference/tracking number</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>High, Medium, or Low (default: Medium)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Job description text</t>
         </is>
       </c>
     </row>
+    <row r="25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -744,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -765,65 +783,70 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Job ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>Client Name</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Job Title</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>State/Region</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Job Function</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Workplace Type</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Application Method</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Job URL</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Reference Number</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -832,65 +855,70 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>JOB-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
           <t>Taskify</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>New York</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Easy Apply</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>https://example.com/job1</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>REF-001</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Full stack role...</t>
         </is>
@@ -899,65 +927,70 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>JOB-002</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
           <t>Taskify</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Data Analyst</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>MH</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Data Analytics</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Easy Apply</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>https://example.com/job2</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>REF-002</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Analytics role...</t>
         </is>
@@ -966,61 +999,66 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>JOB-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
           <t>QuikHire</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>District Manager</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Management</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>ATS</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>https://example.com/job3</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>REF-003</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Retail management...</t>
         </is>
@@ -1029,65 +1067,70 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>JOB-004</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
           <t>QuikHire</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Registered Nurse</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Houston</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Hospitals and Health Care</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>ATS</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>https://example.com/job4</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>REF-004</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Clinical nursing...</t>
         </is>
@@ -1096,61 +1139,66 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>JOB-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
           <t>AI Jobs</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>DevOps Engineer</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Berlin</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Software Development</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Easy Apply</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>https://example.com/job5</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>REF-005</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Cloud infrastructure...</t>
         </is>

</xml_diff>

<commit_message>
S42: Rename Job ID -> Job ID / Project ID in template
Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/data/slotops_upload_template.xlsx
+++ b/data/slotops_upload_template.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Job ID</t>
+          <t>Job ID / Project ID</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unique job identifier (e.g., JOB-001, LinkedIn Job ID). Auto-generated if blank.</t>
+          <t>Unique job or project identifier (e.g., JOB-001, LinkedIn Job ID, Project ID). Auto-generated if blank.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -762,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -783,7 +782,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Job ID</t>
+          <t>Job ID / Project ID</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">

</xml_diff>

<commit_message>
S42: Rename to Project ID
Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/data/slotops_upload_template.xlsx
+++ b/data/slotops_upload_template.xlsx
@@ -515,7 +515,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Job ID / Project ID</t>
+          <t>Project ID</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Job ID / Project ID</t>
+          <t>Project ID</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">

</xml_diff>